<commit_message>
Add Tier A dossier: camerale data, revenue verdicts, public contacts
Approfondimento sui 14 target Tier A: ragione sociale/forma giuridica,
P.IVA, fatturato dove reperibile con verdetto ICP, e recapiti pubblici
(tel/email/PEC/LinkedIn). Nuovo foglio 'Tier A - Dossier' nell'xlsx +
sezione dedicata nella sintesi. Corretta anagrafica Ercoli (SRL in
liquidazione). Lusha senza copertura sui micro-studi: contatti da web.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016SSkfrMp48Szd2c5nWLB3w
</commit_message>
<xml_diff>
--- a/venere-target-search/output/Venere_Longlist_Target.xlsx
+++ b/venere-target-search/output/Venere_Longlist_Target.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Longlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sintesi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ICP e Metodo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Candidati minori" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Esclusi" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tier A - Dossier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sintesi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ICP e Metodo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Candidati minori" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Esclusi" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Longlist'!$A$1:$N$79</definedName>
@@ -121,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -140,6 +141,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -4911,7 +4921,7 @@
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>Dott.ssa Mariangela Ercoli (Mariangela Ercoli S.r.l.)</t>
+          <t>Dott.ssa Mariangela Ercoli (studio prof.; 'Mariangela Ercoli Srl' risulta IN LIQUIDAZIONE)</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
@@ -4926,7 +4936,7 @@
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>Segnale uscita generazionale piu netto: attivo 40+ anni, fondatrice storica, zona premium Parioli, entita SRL propria</t>
+          <t>Fondatrice storica 40+ anni, Parioli premium; MA assetto societario da chiarire (SRL in liquidazione + doppia identita web mariangelaercoli.com / montipariolimedical.it). Attenzione omonimia 'Monti Parioli Medical' (Del Parco)</t>
         </is>
       </c>
       <c r="N61" s="3" t="inlineStr">
@@ -6238,6 +6248,1040 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clinica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ragione sociale / Forma giuridica</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>P.IVA</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Fatturato (anno / fonte)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verdetto ICP EUR 0,8-2,5M</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Telefono</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PEC</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Indirizzo</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Flag / caveat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Studio Medico Estetico Monti Parioli</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Studio prof. / ditta indiv.; 'Mariangela Ercoli Srl' IN LIQUIDAZIONE</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Mariangela Ercoli</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>06 87089918 / 351 4676449 (sito attuale); 06 3226547 (reg.)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>info@montipariolimedical.it</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Via dei Monti Parioli 36, 00197 Roma</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Assetto societario da chiarire: SRL in liquidazione + doppia identita web. Omonimia con 'Monti Parioli Medical' (sorelle Del Parco)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Studio Saccomanno / SabaMedica</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>SAN SABA MEDICA S.R.L. (ATECO 86.22.09)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>fascia EUR 0,3-0,6M (2023) - informazione-aziende.it</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Probabile SOTTO</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Karin Saccomanno</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>06 5757308 / 349 7391039</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>st.saccomanno@gmail.com</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Viale Piramide Cestia 1, 00153 Roma</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Possibile upside se sommato il fatturato su P.IVA personale della dottoressa (non consolidato)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Centro Medico Estetico Raffaella Casilli</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Studio prof. / ditta indiv. (nessuna SRL)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Probabile SOTTO</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Raffaella Casilli</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>06 3220030 / 366 1914536</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>info@raffaellacasilli.com</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/dottoressa-raffaella-casilli</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Viale Belle Arti 7, 00196 Roma (+ Anzio)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Struttura mono-professionale su 2 studi (appuntamento)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Clinica Gramsci</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Firenze/Prato</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CLINICA GRAMSCI - CHIRURGIA PLASTICA E MEDICINA ESTETICA S.R.L.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>07363720488</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>n/d (SRL con bilancio depositato - non accessibile via web)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>n/d - PRIORITARIA visura</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Serena Ghezzi / Dr. Fabio Quercioli</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>055 8358297</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>info@clinicagramsci.it</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>n/d (esiste, non esposta)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/dott-serenaghezzi ; linkedin.com/in/fabio-quercioli-9319b042</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Viale Gramsci 63/65, Firenze (+ V.le Marconi 50/7, Prato)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Unica vera SRL strutturata con bilancio tra i Tier A Roma-Centro: prioritaria per visura camerale a pagamento (i numeri esistono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>JFK Medical Beauty</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Pescara/Perugia</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Non identificata (nessuna 'JFK Srl' confermata)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>n/d (Dr. Carlo Carusi, chirurgo)</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>085 2010818</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>info@jfkmedicalbeauty.it</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Viale J.F. Kennedy 167, 65123 Pescara; Perugia n/d</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Ragione sociale mancante; discordanza indirizzo Pescara (Kennedy 167 vs 'via Bologna'); NON usare 'JMJ Pescara Srls' (non provato il legame)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Poliambulatorio Filippini</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Brescia</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Studio / ditta indiv. (probabile)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>03017310172</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Prof. Enrico Filippini</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>030 2807547 / 335 5850800 / WA 389 2681259</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>info@studiomedicofilippini.it</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/poliambulatoriofilippini (aziendale)</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Via San Francesco d'Assisi 3, 25122 Brescia</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>OMONIMIA: 'Poliambulatorio Filippini S.R.L.' P.IVA 02584010124 e' a Tradate (VA) - entita DIVERSA, non confondere</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Poliambulatorio Finazzi</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Bergamo</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>POLIAMBULATORIO FINAZZI SRL (cost. 2023)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>04697570168</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>EUR 191.671 (2024); 17.580 (2023); 3 dip - reportaziende.it</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Probabile SOTTO</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Glauco Finazzi (AD)</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>035 0770751 / 340 2706511</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>info@poliambulatoriofinazzi.it</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>n/d (esiste, oscurata)</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>it.linkedin.com/in/glauco-finazzi</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Via G.B. Berizzi 45, 24126 Bergamo</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>SRL neocostituita/piccola: se il business reale e' piu' grande il fatturato storico e' probabilmente in un'altra entita' - verificare</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Poliambulatorio Medivela</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>MEDIVELA S.R.L. (cost. 2011, ATECO 86.22.09)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>10020590013</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>EUR 684k (2022) -&gt; 757k (2023) -&gt; ~826k (2024 stima); 4 dip - reportaziende.it/ufficiocamerale</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>DENTRO (borderline floor)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Sergio Periotto (dir. san.)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>011 5612296</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>info@medivela.com</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>medivela.srl@legalmail.it</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Via Vincenzo Vela 2, 10128 Torino</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>UNICO target Tier A con ricavi verificati vicino/dentro la soglia ICP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Clinica Visage</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Genova/Ventimiglia</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Ditta indiv. / studio (ragione sociale non confermata)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>02425900996 (non verificata)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>n/d (dir. san./titolare non pubblico)</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>342 1915957 (anche WhatsApp)</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>info@clinicavisage.it</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Via Ruffini 10/3, 18039 Ventimiglia; Genova (P.za De Ferrari, non confermato)</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Possibile distinzione tra clinicavisage.it e 'Visage Medicina e Chir. Estetica' (P.za Piccapietra 73 Genova, 010 663351) - verificare se stessa struttura. Omonimia 'Visage Srl' San Vitaliano (NA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Medical Laser Clinic</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Verona</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>MEDICAL LASER CLINIC S.R.L. (cost. 2014, ATECO 86.22.06)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>04268200237</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>n/d (SRL con bilancio - non accessibile via web)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Stefano Anderluzzi (+ Dr. Francesco Colla)</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>045 990465 / 371 1457873</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>info@medicallaserclinic.it</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Via Archimede 10, 37036 San Martino B.A. (VR)</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>NON confondere con 'MD Clinic Srl' (04557910231, diagnostica): il fatturato EUR 174k spesso associato via motori e' di MD Clinic, non del target</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>AES Clinic</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Padova</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>PERLA MEDICINA S.R.L. (socio unico, REA PD-447230)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>05153050280</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>n/d (SRL con bilancio - non accessibile via web)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>n/d - miglior candidata al range</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa MianMian Wang</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>049 5225283 / 334 9444309</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>n/d (solo form sul sito)</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>perlamedicina@pec.it</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Sede legale Via del Cristo 378, 35127 Padova; operativa P.le Stazione 7</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>La piu' 'aziendalizzata': SRL/poliambulatorio strutturato. Da chiudere il fatturato con visura CCIAA/Atoka</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Centro San Prospero</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Operatore da identificare ('San Prospero Srl' e' IN LIQUIDAZIONE e ad altro indirizzo)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Antonio Gotti</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>051 0935313 / WA 349 3684962</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>info@medicinaesteticasanprospero.it</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Via Cesare Battisti 2/D-4/A, 40123 Bologna</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Identificare la ragione sociale operativa reale (via C. Battisti 2/D) prima della visura: la 'San Prospero Srl' nota e' vecchio veicolo/omonimia</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Studio Dott.ssa Clelia Barini</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Modena/Formigine</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Studio prof. individuale (dal 1994)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>n/d (snippet discordanti)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Probabile SOTTO</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Clelia Barini</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>059 557249 / 366 1391885</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>info@medicinaesteticabarini.it (+ dottcleliabarini@gmail.com)</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Via G. Pascoli 171, 41043 Corlo di Formigine (MO) (+ La Spezia)</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Studio individuale: fatturato non depositato. Docente Master Med. Estetica UniMoRe, CDA SIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Studio Dott.ssa Paola Molinari</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Modena</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Studio prof. individuale (dal 1987; OMCeO MO n.4036)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>01784820365</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>n/d (non depositato)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Dott.ssa Paola Molinari</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>059 218866 / 333 2472754</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>medicinaesteticamolinari@gmail.com</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>paola.molinari.ospa@mo.omceo.it</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Via Pietro Giardini 45, 41124 Modena</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Studio individuale: fatturato non depositato. Teoxane Training Center, Comitato Scientifico SIES</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6253,21 +7297,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>PROGETTO VENERE - Longlist target medicina estetica (Italia)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Buy-and-build: consolidamento della medicina estetica IT. Deliverable di origination - 26/07/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Copertura</t>
         </is>
@@ -6279,7 +7323,7 @@
           <t>Totale target in longlist</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="13" t="n">
         <v>78</v>
       </c>
     </row>
@@ -6324,7 +7368,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Tiering</t>
         </is>
@@ -6361,351 +7405,351 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>TOP 12 (Tier A) - priorita di approccio</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Clinica</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Citta</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Angolo</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Perche</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Poliambulatorio Medico Chirurgico Filippini</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Brescia (BS)</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>MP+GEN</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Multi-provider affermato + fondatore maturo (uscita generazionale), bacino Brescia ~200k</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Poliambulatorio Finazzi</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Bergamo (BG)</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>MP+GEN+PLAT</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Realta familiare 2 sedi, laser dagli anni '90, dinamica di successione familiare</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Poliambulatorio Medivela</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Torino (Crocetta) (TO)</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>MP+PLAT</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Poliambulatorio strutturato/istituzionalizzato, non dipende da un nome: piattaforma-anchor Torino</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Clinica Visage</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Genova (+ Ventimiglia) (GE)</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>MP+PLAT</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Multi-sede locale affermata, posizionamento rigenerativa/longevity moderno, baricentro Genova</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Medical Laser Clinic</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>San Martino B.A. (Verona) (VR)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Multi-provider indipendente, 2 soci medici, mix laser+iniettabili+derma, bacino Verona</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>AES Clinic (Perla Medicina Srl)</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Padova (PD)</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Profilo piu vicino all'ICP puro: indipendente, multi-provider, non-chirurgico, centro Padova</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Centro San Prospero - Med. e Chir. Estetica</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Bologna (BO)</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Multi-provider indipendente maturo (chir. plastico, medico estetico, derma, flebologo, dietista), hub Bologna</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Studio Dott.ssa Clelia Barini</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Modena (Formigine) (MO)</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>GEN+PLAT</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>Segnale generazionale forte (30 anni, consiglio SIES, docente UniMoRe), multi-sede + energy-based</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Studio Dott.ssa Paola Molinari</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Modena (MO)</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>GEN</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Candidata succession di prim'ordine: 30+ anni, Teoxane Training Center, docente; brand trasferibile</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Studio Medico Estetico Monti Parioli</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Roma (RM)</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>MP+GEN</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Segnale uscita generazionale piu netto: attivo 40+ anni, fondatrice storica, zona premium Parioli, entita SRL propria</t>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Fondatrice storica 40+ anni, Parioli premium; MA assetto societario da chiarire (SRL in liquidazione + doppia identita web mariangelaercoli.com / montipariolimedical.it). Attenzione omonimia 'Monti Parioli Medical' (Del Parco)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Studio Saccomanno / SabaMedica Longevity HUB</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Roma (RM)</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>MP+PLAT</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Indipendente per vocazione (titolare presiede Assoc. Sanita Indipendente), 2 sedi, brand premium</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Centro Medico Estetico Raffaella Casilli</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Roma (+ Anzio) (RM)</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>GEN+PLAT</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>30 anni di esperienza (generazionale), 2 sedi, mix iniettabili + energy-based ripetibili</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Clinica Gramsci - Med. e Chirurgia Estetica</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Firenze / Prato (FI)</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>MP+PLAT</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Gia rete 2 sedi con divisioni distinte estetica/rigenerativa/laser, entita P.IVA dedicata; piattaforma toscana</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>JFK Medical Beauty</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Pescara / Perugia (PE)</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>MP+PLAT</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Rete interregionale gia impostata, core iniettabili ripetibili: mini-piattaforma Abruzzo+Umbria</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Legenda 'Angolo'</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
@@ -6717,7 +7761,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>GEN</t>
         </is>
@@ -6729,7 +7773,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>PLAT</t>
         </is>
@@ -6741,7 +7785,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>CONV</t>
         </is>
@@ -6757,7 +7801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6770,125 +7814,125 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Criteri del target ideale (dal deck Venere, pag. 9)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>- Ricavi EUR 0,8-2,5M, EBITDA margin 20%+ (verificato in DD con normalizzazione ricavi)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>- Citta con bacino 100k+ abitanti; priorita cluster Nord-Ovest, Nord-Est, Roma</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>- Base pazienti attiva 1.500+, prevalenza iniettabili/trattamenti ripetibili</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>- 2+ medici operativi, o struttura convertibile a multi-provider entro 12 mesi</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>- Titolare disponibile a permanenza clinica 24-36 mesi con earn-out e rollover</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>- Autorizzazioni sanitarie in regola e sede idonea all'ampliamento</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr"/>
+      <c r="A8" s="17" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Struttura tipo dell'operazione</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>- Prezzo d'ingresso 3-4x EBITDA normalizzato</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>- 60-70% cash al closing, 15-20% earn-out a 24 mesi, 15-25% rollover equity</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr"/>
+      <c r="A12" s="17" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Metodo di ricerca e limiti</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>- Longlist costruita via ricerca web su 4 cluster (Lombardia; Piemonte-Liguria; Nord-Est; Roma-Centro).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>- Ogni clinica e reale e con fonte URL. Le realta franchising/PE/catene sono state escluse (vedi foglio Esclusi).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>- IMPORTANTE: ricavi ed EBITDA NON sono pubblici per questi studi/SRL privati -&gt; per tutti valgono 'n/d - stima'.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>- Prossimo step: pull camerale (visure/bilanci Registro Imprese) sulle SRL identificate per stimare fatturato vs soglia ICP,</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  ed enrichment dei contatti dei titolari (es. via Lusha) sui Tier A prima dell'approccio.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>- Le autorizzazioni sanitarie regionali vanno confermate puntualmente in due diligence.</t>
         </is>
@@ -6899,7 +7943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6919,42 +7963,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Cluster</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Regione</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="19" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="19" t="inlineStr">
         <is>
           <t>Citta</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="19" t="inlineStr">
         <is>
           <t>Prov</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="19" t="inlineStr">
         <is>
           <t>Sito</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="19" t="inlineStr">
         <is>
           <t>Servizi</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="19" t="inlineStr">
         <is>
           <t>Note (fit debole)</t>
         </is>
@@ -7133,7 +8177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7149,22 +8193,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Cosa e</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="19" t="inlineStr">
         <is>
           <t>Motivo esclusione</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="19" t="inlineStr">
         <is>
           <t>Fonte</t>
         </is>

</xml_diff>